<commit_message>
upload of final files
</commit_message>
<xml_diff>
--- a/7_weitere_beispiele/ue_13_textfunktionen.xlsx
+++ b/7_weitere_beispiele/ue_13_textfunktionen.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a08e36333fa8bc9f/excel_20260302/7_weitere_beispiele/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a08e36333fa8bc9f/excel_20260302_ueberarbeitet/7_weitere_beispiele/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="8_{D90AC2A3-CA99-40D3-91B5-960FD0DEC9F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F54BC6BE-24F6-47F8-A95D-13F35DD17C35}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="8_{D90AC2A3-CA99-40D3-91B5-960FD0DEC9F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4C668A59-6360-4A21-94A5-CE3F3C71220B}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4DF5B1BF-F83B-458E-83BE-C58EC586AC23}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="32">
   <si>
     <t>Art</t>
   </si>
@@ -117,15 +117,6 @@
   </si>
   <si>
     <t>Einweg</t>
-  </si>
-  <si>
-    <t>- 1. Buchstabe der Artikelart (Papier, Haftnotizen, etc.)</t>
-  </si>
-  <si>
-    <t>- 2. die ersten beiden Buchstaben der Herstellerfirma</t>
-  </si>
-  <si>
-    <t>- 3. die volle Bezeichnung des Artikels</t>
   </si>
   <si>
     <r>
@@ -140,6 +131,18 @@
       </rPr>
       <t xml:space="preserve"> Generiere die Artikelnummer wie folgt (jeweils getrennt mit einem Bindestrich):</t>
     </r>
+  </si>
+  <si>
+    <t>- den ersten Buchstaben der Artikelart (Papier, Haftnotizen, etc.)</t>
+  </si>
+  <si>
+    <t>- die ersten beiden Buchstaben der Herstellerfirma</t>
+  </si>
+  <si>
+    <t>- die volle Bezeichnung</t>
+  </si>
+  <si>
+    <t>- die volle Beschreibung</t>
   </si>
 </sst>
 </file>
@@ -668,7 +671,7 @@
       </c>
       <c r="E2" s="5"/>
       <c r="G2" s="9" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -686,7 +689,7 @@
       </c>
       <c r="E3" s="5"/>
       <c r="G3" s="10" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -704,7 +707,7 @@
       </c>
       <c r="E4" s="5"/>
       <c r="G4" s="10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -722,7 +725,7 @@
       </c>
       <c r="E5" s="5"/>
       <c r="G5" s="10" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -739,6 +742,9 @@
         <v>11</v>
       </c>
       <c r="E6" s="5"/>
+      <c r="G6" s="10" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="3" t="s">

</xml_diff>